<commit_message>
changes based on test board manufacturing, mostly added voltage dividers
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dockal\Documents\vut\EPS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAB95DE-DB69-4298-AEB2-D132D0E76CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180F1DAF-A809-474B-831A-B66A97D579B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B25F3AE8-B06D-46FC-8CE9-BDBF7DB59133}"/>
+    <workbookView xWindow="828" yWindow="696" windowWidth="22212" windowHeight="11532" xr2:uid="{B25F3AE8-B06D-46FC-8CE9-BDBF7DB59133}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST_PCB" sheetId="2" r:id="rId1"/>
     <sheet name="List1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">TEST_PCB!$A$1:$F$49</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">TEST_PCB!$A$1:$H$49</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="189">
   <si>
     <t>Reference</t>
   </si>
@@ -176,9 +176,6 @@
     <t>https://cz.mouser.com/datasheet/3/40/1/SRR1260A.pdf</t>
   </si>
   <si>
-    <t>IRLML5103</t>
-  </si>
-  <si>
     <t>Package_TO_SOT_SMD:SOT-23-3</t>
   </si>
   <si>
@@ -449,9 +446,6 @@
     <t>https://cz.mouser.com/ProductDetail/Texas-Instruments/LP38690SD-3.3-NOPB?qs=1FNqv8aZn1Rwc5i1Hgfrsw%3D%3D</t>
   </si>
   <si>
-    <t>https://cz.mouser.com/ProductDetail/Infineon-Technologies/IRLML5103TRPBF?qs=9%252BKlkBgLFf1LjnxxaSUHJw%3D%3D</t>
-  </si>
-  <si>
     <t>Q201,Q301,Q1201</t>
   </si>
   <si>
@@ -495,13 +489,139 @@
   </si>
   <si>
     <t>https://cz.mouser.com/ProductDetail/Panasonic/ERJ-L14UJ20MU?qs=sGAEpiMZZMtlubZbdhIBIKXdPrAL74Yt3W9J5b9tBWs%3D</t>
+  </si>
+  <si>
+    <t>BSS138L</t>
+  </si>
+  <si>
+    <t>https://cz.mouser.com/ProductDetail/onsemi/BSS138L?qs=C8E66ftkQtxfAHmiWaRE%252Bg%3D%3D</t>
+  </si>
+  <si>
+    <t>Sloupec1</t>
+  </si>
+  <si>
+    <t>Mouser MPN</t>
+  </si>
+  <si>
+    <t>512-BSS138L</t>
+  </si>
+  <si>
+    <t>710-830050789</t>
+  </si>
+  <si>
+    <t>595-TCAN4551RGYRQ1</t>
+  </si>
+  <si>
+    <t>595-SP430FR5992IRGZR</t>
+  </si>
+  <si>
+    <t>584-ADG1607BCPZ-R7</t>
+  </si>
+  <si>
+    <t>595-BQ7692000PWR</t>
+  </si>
+  <si>
+    <t>595-TMCS1101A2UQDRQ1</t>
+  </si>
+  <si>
+    <t>926-LM334M/NOPB</t>
+  </si>
+  <si>
+    <t>595-THVD1424RGTR</t>
+  </si>
+  <si>
+    <t>595-LM74700QDBVTQ1</t>
+  </si>
+  <si>
+    <t>595-TPS62933FDRLR</t>
+  </si>
+  <si>
+    <t>595-BQ24650RVAR</t>
+  </si>
+  <si>
+    <t>926-LP38690SD33NOPB</t>
+  </si>
+  <si>
+    <t>594-MCT06030Z0000ZPW</t>
+  </si>
+  <si>
+    <t>667-ERJ-L14UJ20MU</t>
+  </si>
+  <si>
+    <t>71-CRCW060310R0FKEDH</t>
+  </si>
+  <si>
+    <t>https://cz.mouser.com/ProductDetail/Vishay/CRCW060310R0FKEDHP?qs=NE9ChkLHqDkuhGOvoblLsw%3D%3D</t>
+  </si>
+  <si>
+    <t>755-SFR03EZPJ101</t>
+  </si>
+  <si>
+    <t>71-RCA0603100KFKEC</t>
+  </si>
+  <si>
+    <t>603-RC1210JR-070RL</t>
+  </si>
+  <si>
+    <t>652-CR0603-JW-105ELF</t>
+  </si>
+  <si>
+    <t>https://cz.mouser.com/ProductDetail/Bourns/CR0603-JW-105ELF?qs=8H7rU548gMdYcLCrpaOwHw%3D%3D</t>
+  </si>
+  <si>
+    <t>863-VTFWS4D9N04XMTAG</t>
+  </si>
+  <si>
+    <t>652-SRR1260A-6R8Y</t>
+  </si>
+  <si>
+    <t>994-MSS1048T-333MLC</t>
+  </si>
+  <si>
+    <t>595-TPS259802ONRGER</t>
+  </si>
+  <si>
+    <t>595-TPS259830ONRGER</t>
+  </si>
+  <si>
+    <t>78-V8PM104-M3/H</t>
+  </si>
+  <si>
+    <t>187-CL10B334KB8VPNC</t>
+  </si>
+  <si>
+    <t>581-KAF15AR71H102KM</t>
+  </si>
+  <si>
+    <t>581-06035C220JAT2A</t>
+  </si>
+  <si>
+    <t>81-GCM188R71H103KA7J</t>
+  </si>
+  <si>
+    <t>187-CL31B106KBHNNNE</t>
+  </si>
+  <si>
+    <t>603-CC603JRX7R9BB104</t>
+  </si>
+  <si>
+    <t>810-C1608X7R1H105K08</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>neobjednanno</t>
+  </si>
+  <si>
+    <t>xx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -517,6 +637,20 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF212529"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -541,16 +675,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hypertextový odkaz" xfId="1" builtinId="8"/>
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -559,6 +695,22 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -581,11 +733,13 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{60185ED0-0FDC-421B-9367-E64F7ADEC89F}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="9">
-    <queryTableFields count="6">
+  <queryTableRefresh nextId="11">
+    <queryTableFields count="8">
       <queryTableField id="1" name="Reference" tableColumnId="1"/>
       <queryTableField id="2" name="Qty" tableColumnId="2"/>
+      <queryTableField id="10" dataBound="0" tableColumnId="9"/>
       <queryTableField id="3" name="Value" tableColumnId="3"/>
+      <queryTableField id="9" dataBound="0" tableColumnId="5"/>
       <queryTableField id="4" name="DNP" tableColumnId="4"/>
       <queryTableField id="7" name="Footprint" tableColumnId="7"/>
       <queryTableField id="8" name="Datasheet" tableColumnId="8"/>
@@ -599,12 +753,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{26D9A7E8-47BE-42B0-A84F-1B161ECF7926}" name="TEST_PCB" displayName="TEST_PCB" ref="A1:F49" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:F49" xr:uid="{26D9A7E8-47BE-42B0-A84F-1B161ECF7926}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{94A36659-B93F-429C-B0C4-4330E82B202A}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{26D9A7E8-47BE-42B0-A84F-1B161ECF7926}" name="TEST_PCB" displayName="TEST_PCB" ref="A1:H49" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:H49" xr:uid="{26D9A7E8-47BE-42B0-A84F-1B161ECF7926}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{94A36659-B93F-429C-B0C4-4330E82B202A}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{7A1ED906-2A75-4A21-9CF3-EEE08B64927D}" uniqueName="2" name="Qty" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{42CE74DB-FF8A-4F38-B6F3-1D8E1D970806}" uniqueName="3" name="Value" queryTableFieldId="3" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{7AFC57FF-DFFE-4700-9BAE-F48D8B4D57DD}" uniqueName="9" name="Sloupec1" queryTableFieldId="10"/>
+    <tableColumn id="3" xr3:uid="{42CE74DB-FF8A-4F38-B6F3-1D8E1D970806}" uniqueName="3" name="Value" queryTableFieldId="3" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{97F7E06E-E3F7-4E7A-BEB7-93CBD81A4BDD}" uniqueName="5" name="Mouser MPN" queryTableFieldId="9" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{8B3113A8-781C-431F-81E5-A1A4AB75E57A}" uniqueName="4" name="DNP" queryTableFieldId="4" dataDxfId="2"/>
     <tableColumn id="7" xr3:uid="{35D0D64A-758F-467C-BF8B-5801CDC2FE99}" uniqueName="7" name="Footprint" queryTableFieldId="7" dataDxfId="1"/>
     <tableColumn id="8" xr3:uid="{D81996A7-F5CF-4DC5-8E47-B7FEB6A33548}" uniqueName="8" name="Datasheet" queryTableFieldId="8" dataDxfId="0"/>
@@ -930,18 +1086,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06174F2B-BAD1-4C45-80CE-6C6C39435722}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="80.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
     <col min="2" max="2" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="80.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="136.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" customWidth="1"/>
+    <col min="8" max="8" width="136.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -949,985 +1107,1237 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2">
         <v>83</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="H2" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3">
         <v>44</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>141</v>
       </c>
       <c r="B4">
         <v>25</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="H4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="H5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="H6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
+        <v>188</v>
+      </c>
+      <c r="D8" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D9" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="H9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>24</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="H10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>26</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
+        <v>188</v>
+      </c>
+      <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="E11" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="F11" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="H11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>28</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
+        <v>187</v>
+      </c>
+      <c r="D12" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="H12" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>31</v>
       </c>
       <c r="B13">
         <v>8</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
+        <v>188</v>
+      </c>
+      <c r="D13" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G13" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="H13" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>34</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F14" t="s">
+        <v>6</v>
+      </c>
+      <c r="G14" t="s">
         <v>36</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="H14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>38</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
+        <v>186</v>
+      </c>
+      <c r="D15" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" t="s">
+        <v>6</v>
+      </c>
+      <c r="G15" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>134</v>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>132</v>
       </c>
       <c r="B16">
         <v>3</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" t="s">
+        <v>6</v>
+      </c>
+      <c r="G16" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="1" t="s">
+      <c r="H16" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>43</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="B17">
         <v>16</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
+        <v>188</v>
+      </c>
+      <c r="D17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="H17" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>46</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="B18">
         <v>5</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
+        <v>188</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="F18" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="H18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>49</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D19" t="s">
         <v>50</v>
       </c>
-      <c r="B19">
-        <v>6</v>
-      </c>
-      <c r="C19" s="1" t="s">
+      <c r="E19" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F19" t="s">
+        <v>6</v>
+      </c>
+      <c r="G19" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="H19" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>52</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="B20">
         <v>35</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
+        <v>186</v>
+      </c>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F20" t="s">
+        <v>6</v>
+      </c>
+      <c r="G20" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>54</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="B21">
         <v>12</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
+        <v>188</v>
+      </c>
+      <c r="D21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" t="s">
+        <v>51</v>
+      </c>
+      <c r="H21" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>56</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F22" t="s">
+        <v>6</v>
+      </c>
+      <c r="G22" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>58</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F23" t="s">
+        <v>6</v>
+      </c>
+      <c r="G23" t="s">
+        <v>51</v>
+      </c>
+      <c r="H23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>60</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" t="s">
+        <v>6</v>
+      </c>
+      <c r="G24" t="s">
+        <v>51</v>
+      </c>
+      <c r="H24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>62</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F25" t="s">
+        <v>6</v>
+      </c>
+      <c r="G25" t="s">
+        <v>51</v>
+      </c>
+      <c r="H25" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="B26">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>186</v>
+      </c>
+      <c r="D26" t="s">
         <v>65</v>
       </c>
-      <c r="B26">
-        <v>7</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="E26" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="F26" t="s">
+        <v>6</v>
+      </c>
+      <c r="G26" t="s">
+        <v>51</v>
+      </c>
+      <c r="H26" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>66</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="B27">
         <v>2</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
+        <v>188</v>
+      </c>
+      <c r="D27" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G27" t="s">
+        <v>48</v>
+      </c>
+      <c r="H27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>68</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="D28" t="s">
+        <v>69</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G28" t="s">
+        <v>51</v>
+      </c>
+      <c r="H28" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>70</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="B29">
         <v>22</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="D29" t="s">
         <v>25</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" t="s">
         <v>3</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>72</v>
+      <c r="G29" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>71</v>
       </c>
       <c r="B30">
         <v>2</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>75</v>
+      <c r="D30" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F30" t="s">
+        <v>6</v>
+      </c>
+      <c r="G30" t="s">
+        <v>51</v>
+      </c>
+      <c r="H30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>74</v>
       </c>
       <c r="B31">
         <v>2</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>138</v>
+      <c r="D31" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G31" t="s">
+        <v>51</v>
+      </c>
+      <c r="H31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>136</v>
       </c>
       <c r="B32">
         <v>2</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>77</v>
+      <c r="D32" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G32" t="s">
+        <v>51</v>
+      </c>
+      <c r="H32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>76</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F33" t="s">
+        <v>6</v>
+      </c>
+      <c r="G33" t="s">
+        <v>51</v>
+      </c>
+      <c r="H33" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
         <v>78</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="B34">
         <v>1</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F34" t="s">
+        <v>6</v>
+      </c>
+      <c r="G34" t="s">
+        <v>51</v>
+      </c>
+      <c r="H34" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>80</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" t="s">
+        <v>81</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F35" t="s">
+        <v>6</v>
+      </c>
+      <c r="G35" t="s">
+        <v>51</v>
+      </c>
+      <c r="H35" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>82</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="B36">
         <v>8</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" t="s">
         <v>25</v>
       </c>
-      <c r="D36" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>142</v>
+      <c r="E36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F36" t="s">
+        <v>6</v>
+      </c>
+      <c r="G36" t="s">
+        <v>51</v>
+      </c>
+      <c r="H36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>140</v>
       </c>
       <c r="B37">
         <v>36</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>84</v>
+      <c r="C37" t="s">
+        <v>186</v>
+      </c>
+      <c r="D37" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="F37" t="s">
+        <v>6</v>
+      </c>
+      <c r="G37" t="s">
+        <v>51</v>
+      </c>
+      <c r="H37" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>83</v>
       </c>
       <c r="B38">
         <v>2</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" t="s">
+        <v>188</v>
+      </c>
+      <c r="D38" t="s">
+        <v>84</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F38" t="s">
+        <v>6</v>
+      </c>
+      <c r="G38" t="s">
         <v>85</v>
       </c>
-      <c r="D38" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E38" s="1" t="s">
+      <c r="H38" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>86</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="B39">
         <v>1</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" t="s">
+        <v>188</v>
+      </c>
+      <c r="D39" t="s">
+        <v>87</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F39" t="s">
+        <v>6</v>
+      </c>
+      <c r="G39" t="s">
         <v>88</v>
       </c>
-      <c r="D39" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E39" s="1" t="s">
+      <c r="H39" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>89</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="B40">
         <v>4</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" t="s">
+        <v>188</v>
+      </c>
+      <c r="D40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F40" t="s">
+        <v>6</v>
+      </c>
+      <c r="G40" t="s">
         <v>91</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E40" s="1" t="s">
+      <c r="H40" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>92</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="B41">
         <v>10</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" t="s">
+        <v>188</v>
+      </c>
+      <c r="D41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F41" t="s">
+        <v>6</v>
+      </c>
+      <c r="G41" t="s">
         <v>94</v>
       </c>
-      <c r="D41" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E41" s="1" t="s">
+      <c r="H41" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>95</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" t="s">
+        <v>188</v>
+      </c>
+      <c r="D42" t="s">
+        <v>96</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F42" t="s">
+        <v>6</v>
+      </c>
+      <c r="G42" t="s">
         <v>97</v>
       </c>
-      <c r="D42" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E42" s="1" t="s">
+      <c r="H42" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>98</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" t="s">
+        <v>188</v>
+      </c>
+      <c r="D43" t="s">
+        <v>99</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F43" t="s">
+        <v>6</v>
+      </c>
+      <c r="G43" t="s">
         <v>100</v>
       </c>
-      <c r="D43" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E43" s="1" t="s">
+      <c r="H43" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>101</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="B44">
         <v>3</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" t="s">
+        <v>188</v>
+      </c>
+      <c r="D44" t="s">
+        <v>102</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F44" t="s">
+        <v>6</v>
+      </c>
+      <c r="G44" t="s">
+        <v>100</v>
+      </c>
+      <c r="H44" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>103</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="B45">
         <v>1</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" t="s">
+        <v>188</v>
+      </c>
+      <c r="D45" t="s">
+        <v>104</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F45" t="s">
+        <v>6</v>
+      </c>
+      <c r="G45" t="s">
         <v>105</v>
       </c>
-      <c r="D45" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E45" s="1" t="s">
+      <c r="H45" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
         <v>106</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="B46">
         <v>1</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" t="s">
+        <v>188</v>
+      </c>
+      <c r="D46" t="s">
+        <v>107</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F46" t="s">
+        <v>6</v>
+      </c>
+      <c r="G46" t="s">
         <v>108</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E46" s="1" t="s">
+      <c r="H46" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>109</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="B47">
         <v>2</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" t="s">
+        <v>188</v>
+      </c>
+      <c r="D47" t="s">
+        <v>110</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F47" t="s">
+        <v>6</v>
+      </c>
+      <c r="G47" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E47" s="1" t="s">
+      <c r="H47" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
         <v>112</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" t="s">
+        <v>188</v>
+      </c>
+      <c r="D48" t="s">
+        <v>113</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F48" t="s">
+        <v>6</v>
+      </c>
+      <c r="G48" t="s">
         <v>114</v>
       </c>
-      <c r="D48" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E48" s="1" t="s">
+      <c r="H48" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>115</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="B49">
         <v>2</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" t="s">
+        <v>188</v>
+      </c>
+      <c r="D49" t="s">
+        <v>116</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F49" t="s">
+        <v>6</v>
+      </c>
+      <c r="G49" t="s">
         <v>117</v>
       </c>
-      <c r="D49" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>123</v>
+      <c r="H49" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{1E1B97B8-70CA-450B-9596-E2034361F13F}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{1E1B97B8-70CA-450B-9596-E2034361F13F}"/>
+    <hyperlink ref="H15" r:id="rId2" xr:uid="{C8A53F28-4153-494C-AD81-914592E68F27}"/>
+    <hyperlink ref="H13" r:id="rId3" xr:uid="{93EAE2EE-6AB9-4D50-8CCF-A74F0469DA85}"/>
+    <hyperlink ref="H47" r:id="rId4" xr:uid="{A31CFFAC-AB29-49BF-92DD-292C13409F47}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
small changes to test board
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dockal\Documents\vut\EPS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180F1DAF-A809-474B-831A-B66A97D579B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E58433-5B96-4768-9E6A-970056C3C975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="828" yWindow="696" windowWidth="22212" windowHeight="11532" xr2:uid="{B25F3AE8-B06D-46FC-8CE9-BDBF7DB59133}"/>
   </bookViews>
@@ -2220,7 +2220,7 @@
       <c r="G45" t="s">
         <v>105</v>
       </c>
-      <c r="H45" t="s">
+      <c r="H45" s="4" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2334,10 +2334,11 @@
     <hyperlink ref="H15" r:id="rId2" xr:uid="{C8A53F28-4153-494C-AD81-914592E68F27}"/>
     <hyperlink ref="H13" r:id="rId3" xr:uid="{93EAE2EE-6AB9-4D50-8CCF-A74F0469DA85}"/>
     <hyperlink ref="H47" r:id="rId4" xr:uid="{A31CFFAC-AB29-49BF-92DD-292C13409F47}"/>
+    <hyperlink ref="H45" r:id="rId5" xr:uid="{72D305C6-EA27-4D82-B7BC-814743D0CB49}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>